<commit_message>
Add telefone and disclaimer to signature generation
- Updated SignatureHTML and SignatureImage classes to include telefone.
- Enhanced carregar_pessoas function to return telefone along with cargo.
- Added disclaimer for AFBR Investimentos in the signature.
</commit_message>
<xml_diff>
--- a/cargos.xlsx
+++ b/cargos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ijasenovski/afs_assinaturas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F89A507-E99D-3346-991D-F2776A1F84C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0D6115-0390-7A47-A291-E9109B7CBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3160" yWindow="2220" windowWidth="28240" windowHeight="17240" xr2:uid="{C42CD4E2-3A71-2847-BF3A-AA2520943A2E}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="75">
   <si>
     <t>Nome</t>
   </si>
@@ -155,13 +155,103 @@
   </si>
   <si>
     <t>João Paulo Luque</t>
+  </si>
+  <si>
+    <t>Telefone</t>
+  </si>
+  <si>
+    <t>(48) 99610-8929</t>
+  </si>
+  <si>
+    <t>(11) 95113-0158</t>
+  </si>
+  <si>
+    <t>(48) 99109-0907</t>
+  </si>
+  <si>
+    <t>(11) 98506-4099</t>
+  </si>
+  <si>
+    <t>(11) 97113-8140</t>
+  </si>
+  <si>
+    <t>(11) 96677-4079</t>
+  </si>
+  <si>
+    <t>(11) 99931-6977</t>
+  </si>
+  <si>
+    <t>(11) 97375-6431</t>
+  </si>
+  <si>
+    <t>(11) 96293-6772</t>
+  </si>
+  <si>
+    <t>(11) 97215-6609</t>
+  </si>
+  <si>
+    <t>(11) 98379-6186</t>
+  </si>
+  <si>
+    <t>(19) 99812-9808</t>
+  </si>
+  <si>
+    <t>(44) 99986-6224</t>
+  </si>
+  <si>
+    <t>(11) 99645-0339</t>
+  </si>
+  <si>
+    <t>(11) 98263-0828</t>
+  </si>
+  <si>
+    <t>(11) 99763-9723</t>
+  </si>
+  <si>
+    <t>(11) 98229-9970</t>
+  </si>
+  <si>
+    <t>(11) 98107-6185</t>
+  </si>
+  <si>
+    <t>(11) 99739-6762</t>
+  </si>
+  <si>
+    <t>(11) 99463-8780</t>
+  </si>
+  <si>
+    <t>(11) 96407-4957</t>
+  </si>
+  <si>
+    <t>(11) 94911-6514</t>
+  </si>
+  <si>
+    <t>(11) 98179-7002</t>
+  </si>
+  <si>
+    <t>(17) 98132-4999</t>
+  </si>
+  <si>
+    <t>(11) 95334-2569</t>
+  </si>
+  <si>
+    <t>(11) 99852-1810</t>
+  </si>
+  <si>
+    <t>(11) 97229-8044</t>
+  </si>
+  <si>
+    <t>(11) 95841-9816</t>
+  </si>
+  <si>
+    <t>(48) 99167-5547</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -295,6 +385,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -638,8 +734,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1015,251 +1112,342 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A7B146-64E0-984C-8919-1D445D5873E4}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C3" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C7" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C8" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>11</v>
       </c>
       <c r="B9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C9" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>12</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C10" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C11" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>14</v>
       </c>
       <c r="B12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C12" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>42</v>
       </c>
       <c r="B13" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C13" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C14" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>43</v>
       </c>
       <c r="B15" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C15" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>44</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C16" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
       <c r="B17" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C17" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>19</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C18" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>21</v>
       </c>
       <c r="B19" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C19" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>23</v>
       </c>
       <c r="B20" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C20" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>25</v>
       </c>
       <c r="B21" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C21" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>26</v>
       </c>
       <c r="B22" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C22" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>27</v>
       </c>
       <c r="B23" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C23" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>28</v>
       </c>
       <c r="B24" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C24" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>29</v>
       </c>
       <c r="B25" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C25" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>31</v>
       </c>
       <c r="B26" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C26" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>32</v>
       </c>
       <c r="B27" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C27" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>33</v>
       </c>
       <c r="B28" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C28" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>34</v>
       </c>
       <c r="B29" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C29" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>36</v>
       </c>
       <c r="B30" t="s">
         <v>37</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add disclaimer for Amazonia Innovation Funding and update signature generation logic
</commit_message>
<xml_diff>
--- a/cargos.xlsx
+++ b/cargos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ijasenovski/afs_assinaturas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0D6115-0390-7A47-A291-E9109B7CBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AD2B36-57E6-DC45-AECA-6DB77EBBF418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3160" yWindow="2220" windowWidth="28240" windowHeight="17240" xr2:uid="{C42CD4E2-3A71-2847-BF3A-AA2520943A2E}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="78">
   <si>
     <t>Nome</t>
   </si>
@@ -245,6 +245,15 @@
   </si>
   <si>
     <t>(48) 99167-5547</t>
+  </si>
+  <si>
+    <t>Denis Feitosa</t>
+  </si>
+  <si>
+    <t>(11) 94796-5538</t>
+  </si>
+  <si>
+    <t>Renda Variável</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1121,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49A7B146-64E0-984C-8919-1D445D5873E4}">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -1221,232 +1230,243 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
         <v>38</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
         <v>38</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
         <v>40</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" t="s">
         <v>38</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>36</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>37</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update cargos.xlsx with new data
</commit_message>
<xml_diff>
--- a/cargos.xlsx
+++ b/cargos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ijasenovski/afs_assinaturas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AD2B36-57E6-DC45-AECA-6DB77EBBF418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0549FE3C-C12D-CF46-8387-4975441A9F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3160" yWindow="2220" windowWidth="28240" windowHeight="17240" xr2:uid="{C42CD4E2-3A71-2847-BF3A-AA2520943A2E}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" xr2:uid="{C42CD4E2-3A71-2847-BF3A-AA2520943A2E}"/>
   </bookViews>
   <sheets>
     <sheet name="cargos" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="77">
   <si>
     <t>Nome</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>Alexandra Molina</t>
-  </si>
-  <si>
-    <t>SÛcia</t>
   </si>
   <si>
     <t>Amanda Burd</t>
@@ -1137,7 +1134,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -1145,10 +1142,10 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
@@ -1156,10 +1153,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1167,10 +1164,10 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
@@ -1178,296 +1175,296 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="B10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="B13" t="s">
-        <v>15</v>
-      </c>
       <c r="C13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
         <v>19</v>
       </c>
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
       <c r="C19" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" t="s">
         <v>21</v>
       </c>
-      <c r="B20" t="s">
-        <v>22</v>
-      </c>
       <c r="C20" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
         <v>23</v>
       </c>
-      <c r="B21" t="s">
-        <v>24</v>
-      </c>
       <c r="C21" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" t="s">
         <v>29</v>
       </c>
-      <c r="B26" t="s">
-        <v>30</v>
-      </c>
       <c r="C26" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" t="s">
         <v>34</v>
       </c>
-      <c r="B30" t="s">
-        <v>35</v>
-      </c>
       <c r="C30" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" t="s">
         <v>36</v>
       </c>
-      <c r="B31" t="s">
-        <v>37</v>
-      </c>
       <c r="C31" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>